<commit_message>
feat: Implement client-side cache and acronym matching for autocomplete and hide pricing from doctor dashboard
</commit_message>
<xml_diff>
--- a/Lab_test_db.xlsx
+++ b/Lab_test_db.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\OneDrive\Desktop\CareConnect 2.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2F0DD9D6-5F55-4799-B7F1-BA4FFCE82464}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F7E8EB6-BA69-43B6-AF85-CCDCAC909DA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3111" uniqueCount="1127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3110" uniqueCount="1127">
   <si>
     <t>Test Name</t>
   </si>
@@ -3407,6 +3407,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="8" formatCode="&quot;₹&quot;\ #,##0.00;[Red]&quot;₹&quot;\ \-#,##0.00"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -3442,9 +3445,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="8" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5761,8 +5765,8 @@
       <c r="B190" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C190" s="1" t="s">
-        <v>247</v>
+      <c r="C190" s="2">
+        <v>120</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>